<commit_message>
Auto update RUP 2026-08-10 08:48:51
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-10).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-08-10).xlsx
@@ -560,7 +560,7 @@
         <v>830740630</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>830740630</v>
@@ -572,7 +572,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>830740630</v>
@@ -1226,7 +1226,7 @@
         <v>61655471600</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>9467977800</v>
@@ -1238,7 +1238,7 @@
         <v>52187493800</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>61655471600</v>

</xml_diff>